<commit_message>
Corregir #VALUE! en Ordenes y forzar recalculo al abrir
- Ordenes: las columnas de semana, total de unidades y total en soles
  devolvian #VALUE! en los renglones sin material porque multiplicaban
  un numero por el texto vacio del precio. Ahora quedan en blanco hasta
  que se registre el material en el maestro.
- Se activa fullCalcOnLoad para que Excel recalcule todas las formulas
  al abrir el archivo.

Verificado con evaluacion de las 524 formulas: 0 celdas con error.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KofGASuDqP2DkSsvGxsHDK
</commit_message>
<xml_diff>
--- a/MRP_ATMIN_plantilla.xlsx
+++ b/MRP_ATMIN_plantilla.xlsx
@@ -12037,43 +12037,43 @@
         <v/>
       </c>
       <c r="E5" s="55">
-        <f>MRP!E10</f>
+        <f>IF($A5="","",MRP!E10)</f>
         <v/>
       </c>
       <c r="F5" s="55">
-        <f>MRP!F10</f>
+        <f>IF($A5="","",MRP!F10)</f>
         <v/>
       </c>
       <c r="G5" s="55">
-        <f>MRP!G10</f>
+        <f>IF($A5="","",MRP!G10)</f>
         <v/>
       </c>
       <c r="H5" s="55">
-        <f>MRP!H10</f>
+        <f>IF($A5="","",MRP!H10)</f>
         <v/>
       </c>
       <c r="I5" s="55">
-        <f>MRP!I10</f>
+        <f>IF($A5="","",MRP!I10)</f>
         <v/>
       </c>
       <c r="J5" s="55">
-        <f>MRP!J10</f>
+        <f>IF($A5="","",MRP!J10)</f>
         <v/>
       </c>
       <c r="K5" s="55">
-        <f>MRP!K10</f>
+        <f>IF($A5="","",MRP!K10)</f>
         <v/>
       </c>
       <c r="L5" s="55">
-        <f>MRP!L10</f>
+        <f>IF($A5="","",MRP!L10)</f>
         <v/>
       </c>
       <c r="M5" s="56">
-        <f>SUM(E5:L5)</f>
+        <f>IF($A5="","",SUM(E5:L5))</f>
         <v/>
       </c>
       <c r="N5" s="57">
-        <f>M5*D5</f>
+        <f>IF($A5="","",M5*D5)</f>
         <v/>
       </c>
     </row>
@@ -12095,43 +12095,43 @@
         <v/>
       </c>
       <c r="E6" s="55">
-        <f>MRP!E17</f>
+        <f>IF($A6="","",MRP!E17)</f>
         <v/>
       </c>
       <c r="F6" s="55">
-        <f>MRP!F17</f>
+        <f>IF($A6="","",MRP!F17)</f>
         <v/>
       </c>
       <c r="G6" s="55">
-        <f>MRP!G17</f>
+        <f>IF($A6="","",MRP!G17)</f>
         <v/>
       </c>
       <c r="H6" s="55">
-        <f>MRP!H17</f>
+        <f>IF($A6="","",MRP!H17)</f>
         <v/>
       </c>
       <c r="I6" s="55">
-        <f>MRP!I17</f>
+        <f>IF($A6="","",MRP!I17)</f>
         <v/>
       </c>
       <c r="J6" s="55">
-        <f>MRP!J17</f>
+        <f>IF($A6="","",MRP!J17)</f>
         <v/>
       </c>
       <c r="K6" s="55">
-        <f>MRP!K17</f>
+        <f>IF($A6="","",MRP!K17)</f>
         <v/>
       </c>
       <c r="L6" s="55">
-        <f>MRP!L17</f>
+        <f>IF($A6="","",MRP!L17)</f>
         <v/>
       </c>
       <c r="M6" s="56">
-        <f>SUM(E6:L6)</f>
+        <f>IF($A6="","",SUM(E6:L6))</f>
         <v/>
       </c>
       <c r="N6" s="57">
-        <f>M6*D6</f>
+        <f>IF($A6="","",M6*D6)</f>
         <v/>
       </c>
     </row>
@@ -12153,43 +12153,43 @@
         <v/>
       </c>
       <c r="E7" s="55">
-        <f>MRP!E24</f>
+        <f>IF($A7="","",MRP!E24)</f>
         <v/>
       </c>
       <c r="F7" s="55">
-        <f>MRP!F24</f>
+        <f>IF($A7="","",MRP!F24)</f>
         <v/>
       </c>
       <c r="G7" s="55">
-        <f>MRP!G24</f>
+        <f>IF($A7="","",MRP!G24)</f>
         <v/>
       </c>
       <c r="H7" s="55">
-        <f>MRP!H24</f>
+        <f>IF($A7="","",MRP!H24)</f>
         <v/>
       </c>
       <c r="I7" s="55">
-        <f>MRP!I24</f>
+        <f>IF($A7="","",MRP!I24)</f>
         <v/>
       </c>
       <c r="J7" s="55">
-        <f>MRP!J24</f>
+        <f>IF($A7="","",MRP!J24)</f>
         <v/>
       </c>
       <c r="K7" s="55">
-        <f>MRP!K24</f>
+        <f>IF($A7="","",MRP!K24)</f>
         <v/>
       </c>
       <c r="L7" s="55">
-        <f>MRP!L24</f>
+        <f>IF($A7="","",MRP!L24)</f>
         <v/>
       </c>
       <c r="M7" s="56">
-        <f>SUM(E7:L7)</f>
+        <f>IF($A7="","",SUM(E7:L7))</f>
         <v/>
       </c>
       <c r="N7" s="57">
-        <f>M7*D7</f>
+        <f>IF($A7="","",M7*D7)</f>
         <v/>
       </c>
     </row>
@@ -12211,43 +12211,43 @@
         <v/>
       </c>
       <c r="E8" s="55">
-        <f>MRP!E31</f>
+        <f>IF($A8="","",MRP!E31)</f>
         <v/>
       </c>
       <c r="F8" s="55">
-        <f>MRP!F31</f>
+        <f>IF($A8="","",MRP!F31)</f>
         <v/>
       </c>
       <c r="G8" s="55">
-        <f>MRP!G31</f>
+        <f>IF($A8="","",MRP!G31)</f>
         <v/>
       </c>
       <c r="H8" s="55">
-        <f>MRP!H31</f>
+        <f>IF($A8="","",MRP!H31)</f>
         <v/>
       </c>
       <c r="I8" s="55">
-        <f>MRP!I31</f>
+        <f>IF($A8="","",MRP!I31)</f>
         <v/>
       </c>
       <c r="J8" s="55">
-        <f>MRP!J31</f>
+        <f>IF($A8="","",MRP!J31)</f>
         <v/>
       </c>
       <c r="K8" s="55">
-        <f>MRP!K31</f>
+        <f>IF($A8="","",MRP!K31)</f>
         <v/>
       </c>
       <c r="L8" s="55">
-        <f>MRP!L31</f>
+        <f>IF($A8="","",MRP!L31)</f>
         <v/>
       </c>
       <c r="M8" s="56">
-        <f>SUM(E8:L8)</f>
+        <f>IF($A8="","",SUM(E8:L8))</f>
         <v/>
       </c>
       <c r="N8" s="57">
-        <f>M8*D8</f>
+        <f>IF($A8="","",M8*D8)</f>
         <v/>
       </c>
     </row>
@@ -12269,43 +12269,43 @@
         <v/>
       </c>
       <c r="E9" s="55">
-        <f>MRP!E38</f>
+        <f>IF($A9="","",MRP!E38)</f>
         <v/>
       </c>
       <c r="F9" s="55">
-        <f>MRP!F38</f>
+        <f>IF($A9="","",MRP!F38)</f>
         <v/>
       </c>
       <c r="G9" s="55">
-        <f>MRP!G38</f>
+        <f>IF($A9="","",MRP!G38)</f>
         <v/>
       </c>
       <c r="H9" s="55">
-        <f>MRP!H38</f>
+        <f>IF($A9="","",MRP!H38)</f>
         <v/>
       </c>
       <c r="I9" s="55">
-        <f>MRP!I38</f>
+        <f>IF($A9="","",MRP!I38)</f>
         <v/>
       </c>
       <c r="J9" s="55">
-        <f>MRP!J38</f>
+        <f>IF($A9="","",MRP!J38)</f>
         <v/>
       </c>
       <c r="K9" s="55">
-        <f>MRP!K38</f>
+        <f>IF($A9="","",MRP!K38)</f>
         <v/>
       </c>
       <c r="L9" s="55">
-        <f>MRP!L38</f>
+        <f>IF($A9="","",MRP!L38)</f>
         <v/>
       </c>
       <c r="M9" s="56">
-        <f>SUM(E9:L9)</f>
+        <f>IF($A9="","",SUM(E9:L9))</f>
         <v/>
       </c>
       <c r="N9" s="57">
-        <f>M9*D9</f>
+        <f>IF($A9="","",M9*D9)</f>
         <v/>
       </c>
     </row>
@@ -12327,43 +12327,43 @@
         <v/>
       </c>
       <c r="E10" s="55">
-        <f>MRP!E45</f>
+        <f>IF($A10="","",MRP!E45)</f>
         <v/>
       </c>
       <c r="F10" s="55">
-        <f>MRP!F45</f>
+        <f>IF($A10="","",MRP!F45)</f>
         <v/>
       </c>
       <c r="G10" s="55">
-        <f>MRP!G45</f>
+        <f>IF($A10="","",MRP!G45)</f>
         <v/>
       </c>
       <c r="H10" s="55">
-        <f>MRP!H45</f>
+        <f>IF($A10="","",MRP!H45)</f>
         <v/>
       </c>
       <c r="I10" s="55">
-        <f>MRP!I45</f>
+        <f>IF($A10="","",MRP!I45)</f>
         <v/>
       </c>
       <c r="J10" s="55">
-        <f>MRP!J45</f>
+        <f>IF($A10="","",MRP!J45)</f>
         <v/>
       </c>
       <c r="K10" s="55">
-        <f>MRP!K45</f>
+        <f>IF($A10="","",MRP!K45)</f>
         <v/>
       </c>
       <c r="L10" s="55">
-        <f>MRP!L45</f>
+        <f>IF($A10="","",MRP!L45)</f>
         <v/>
       </c>
       <c r="M10" s="56">
-        <f>SUM(E10:L10)</f>
+        <f>IF($A10="","",SUM(E10:L10))</f>
         <v/>
       </c>
       <c r="N10" s="57">
-        <f>M10*D10</f>
+        <f>IF($A10="","",M10*D10)</f>
         <v/>
       </c>
     </row>
@@ -12385,43 +12385,43 @@
         <v/>
       </c>
       <c r="E11" s="55">
-        <f>MRP!E52</f>
+        <f>IF($A11="","",MRP!E52)</f>
         <v/>
       </c>
       <c r="F11" s="55">
-        <f>MRP!F52</f>
+        <f>IF($A11="","",MRP!F52)</f>
         <v/>
       </c>
       <c r="G11" s="55">
-        <f>MRP!G52</f>
+        <f>IF($A11="","",MRP!G52)</f>
         <v/>
       </c>
       <c r="H11" s="55">
-        <f>MRP!H52</f>
+        <f>IF($A11="","",MRP!H52)</f>
         <v/>
       </c>
       <c r="I11" s="55">
-        <f>MRP!I52</f>
+        <f>IF($A11="","",MRP!I52)</f>
         <v/>
       </c>
       <c r="J11" s="55">
-        <f>MRP!J52</f>
+        <f>IF($A11="","",MRP!J52)</f>
         <v/>
       </c>
       <c r="K11" s="55">
-        <f>MRP!K52</f>
+        <f>IF($A11="","",MRP!K52)</f>
         <v/>
       </c>
       <c r="L11" s="55">
-        <f>MRP!L52</f>
+        <f>IF($A11="","",MRP!L52)</f>
         <v/>
       </c>
       <c r="M11" s="56">
-        <f>SUM(E11:L11)</f>
+        <f>IF($A11="","",SUM(E11:L11))</f>
         <v/>
       </c>
       <c r="N11" s="57">
-        <f>M11*D11</f>
+        <f>IF($A11="","",M11*D11)</f>
         <v/>
       </c>
     </row>
@@ -12443,43 +12443,43 @@
         <v/>
       </c>
       <c r="E12" s="55">
-        <f>MRP!E59</f>
+        <f>IF($A12="","",MRP!E59)</f>
         <v/>
       </c>
       <c r="F12" s="55">
-        <f>MRP!F59</f>
+        <f>IF($A12="","",MRP!F59)</f>
         <v/>
       </c>
       <c r="G12" s="55">
-        <f>MRP!G59</f>
+        <f>IF($A12="","",MRP!G59)</f>
         <v/>
       </c>
       <c r="H12" s="55">
-        <f>MRP!H59</f>
+        <f>IF($A12="","",MRP!H59)</f>
         <v/>
       </c>
       <c r="I12" s="55">
-        <f>MRP!I59</f>
+        <f>IF($A12="","",MRP!I59)</f>
         <v/>
       </c>
       <c r="J12" s="55">
-        <f>MRP!J59</f>
+        <f>IF($A12="","",MRP!J59)</f>
         <v/>
       </c>
       <c r="K12" s="55">
-        <f>MRP!K59</f>
+        <f>IF($A12="","",MRP!K59)</f>
         <v/>
       </c>
       <c r="L12" s="55">
-        <f>MRP!L59</f>
+        <f>IF($A12="","",MRP!L59)</f>
         <v/>
       </c>
       <c r="M12" s="56">
-        <f>SUM(E12:L12)</f>
+        <f>IF($A12="","",SUM(E12:L12))</f>
         <v/>
       </c>
       <c r="N12" s="57">
-        <f>M12*D12</f>
+        <f>IF($A12="","",M12*D12)</f>
         <v/>
       </c>
     </row>
@@ -12501,43 +12501,43 @@
         <v/>
       </c>
       <c r="E13" s="55">
-        <f>MRP!E66</f>
+        <f>IF($A13="","",MRP!E66)</f>
         <v/>
       </c>
       <c r="F13" s="55">
-        <f>MRP!F66</f>
+        <f>IF($A13="","",MRP!F66)</f>
         <v/>
       </c>
       <c r="G13" s="55">
-        <f>MRP!G66</f>
+        <f>IF($A13="","",MRP!G66)</f>
         <v/>
       </c>
       <c r="H13" s="55">
-        <f>MRP!H66</f>
+        <f>IF($A13="","",MRP!H66)</f>
         <v/>
       </c>
       <c r="I13" s="55">
-        <f>MRP!I66</f>
+        <f>IF($A13="","",MRP!I66)</f>
         <v/>
       </c>
       <c r="J13" s="55">
-        <f>MRP!J66</f>
+        <f>IF($A13="","",MRP!J66)</f>
         <v/>
       </c>
       <c r="K13" s="55">
-        <f>MRP!K66</f>
+        <f>IF($A13="","",MRP!K66)</f>
         <v/>
       </c>
       <c r="L13" s="55">
-        <f>MRP!L66</f>
+        <f>IF($A13="","",MRP!L66)</f>
         <v/>
       </c>
       <c r="M13" s="56">
-        <f>SUM(E13:L13)</f>
+        <f>IF($A13="","",SUM(E13:L13))</f>
         <v/>
       </c>
       <c r="N13" s="57">
-        <f>M13*D13</f>
+        <f>IF($A13="","",M13*D13)</f>
         <v/>
       </c>
     </row>
@@ -12559,43 +12559,43 @@
         <v/>
       </c>
       <c r="E14" s="55">
-        <f>MRP!E73</f>
+        <f>IF($A14="","",MRP!E73)</f>
         <v/>
       </c>
       <c r="F14" s="55">
-        <f>MRP!F73</f>
+        <f>IF($A14="","",MRP!F73)</f>
         <v/>
       </c>
       <c r="G14" s="55">
-        <f>MRP!G73</f>
+        <f>IF($A14="","",MRP!G73)</f>
         <v/>
       </c>
       <c r="H14" s="55">
-        <f>MRP!H73</f>
+        <f>IF($A14="","",MRP!H73)</f>
         <v/>
       </c>
       <c r="I14" s="55">
-        <f>MRP!I73</f>
+        <f>IF($A14="","",MRP!I73)</f>
         <v/>
       </c>
       <c r="J14" s="55">
-        <f>MRP!J73</f>
+        <f>IF($A14="","",MRP!J73)</f>
         <v/>
       </c>
       <c r="K14" s="55">
-        <f>MRP!K73</f>
+        <f>IF($A14="","",MRP!K73)</f>
         <v/>
       </c>
       <c r="L14" s="55">
-        <f>MRP!L73</f>
+        <f>IF($A14="","",MRP!L73)</f>
         <v/>
       </c>
       <c r="M14" s="56">
-        <f>SUM(E14:L14)</f>
+        <f>IF($A14="","",SUM(E14:L14))</f>
         <v/>
       </c>
       <c r="N14" s="57">
-        <f>M14*D14</f>
+        <f>IF($A14="","",M14*D14)</f>
         <v/>
       </c>
     </row>
@@ -12617,43 +12617,43 @@
         <v/>
       </c>
       <c r="E15" s="55">
-        <f>MRP!E80</f>
+        <f>IF($A15="","",MRP!E80)</f>
         <v/>
       </c>
       <c r="F15" s="55">
-        <f>MRP!F80</f>
+        <f>IF($A15="","",MRP!F80)</f>
         <v/>
       </c>
       <c r="G15" s="55">
-        <f>MRP!G80</f>
+        <f>IF($A15="","",MRP!G80)</f>
         <v/>
       </c>
       <c r="H15" s="55">
-        <f>MRP!H80</f>
+        <f>IF($A15="","",MRP!H80)</f>
         <v/>
       </c>
       <c r="I15" s="55">
-        <f>MRP!I80</f>
+        <f>IF($A15="","",MRP!I80)</f>
         <v/>
       </c>
       <c r="J15" s="55">
-        <f>MRP!J80</f>
+        <f>IF($A15="","",MRP!J80)</f>
         <v/>
       </c>
       <c r="K15" s="55">
-        <f>MRP!K80</f>
+        <f>IF($A15="","",MRP!K80)</f>
         <v/>
       </c>
       <c r="L15" s="55">
-        <f>MRP!L80</f>
+        <f>IF($A15="","",MRP!L80)</f>
         <v/>
       </c>
       <c r="M15" s="56">
-        <f>SUM(E15:L15)</f>
+        <f>IF($A15="","",SUM(E15:L15))</f>
         <v/>
       </c>
       <c r="N15" s="57">
-        <f>M15*D15</f>
+        <f>IF($A15="","",M15*D15)</f>
         <v/>
       </c>
     </row>
@@ -12675,43 +12675,43 @@
         <v/>
       </c>
       <c r="E16" s="55">
-        <f>MRP!E87</f>
+        <f>IF($A16="","",MRP!E87)</f>
         <v/>
       </c>
       <c r="F16" s="55">
-        <f>MRP!F87</f>
+        <f>IF($A16="","",MRP!F87)</f>
         <v/>
       </c>
       <c r="G16" s="55">
-        <f>MRP!G87</f>
+        <f>IF($A16="","",MRP!G87)</f>
         <v/>
       </c>
       <c r="H16" s="55">
-        <f>MRP!H87</f>
+        <f>IF($A16="","",MRP!H87)</f>
         <v/>
       </c>
       <c r="I16" s="55">
-        <f>MRP!I87</f>
+        <f>IF($A16="","",MRP!I87)</f>
         <v/>
       </c>
       <c r="J16" s="55">
-        <f>MRP!J87</f>
+        <f>IF($A16="","",MRP!J87)</f>
         <v/>
       </c>
       <c r="K16" s="55">
-        <f>MRP!K87</f>
+        <f>IF($A16="","",MRP!K87)</f>
         <v/>
       </c>
       <c r="L16" s="55">
-        <f>MRP!L87</f>
+        <f>IF($A16="","",MRP!L87)</f>
         <v/>
       </c>
       <c r="M16" s="56">
-        <f>SUM(E16:L16)</f>
+        <f>IF($A16="","",SUM(E16:L16))</f>
         <v/>
       </c>
       <c r="N16" s="57">
-        <f>M16*D16</f>
+        <f>IF($A16="","",M16*D16)</f>
         <v/>
       </c>
     </row>
@@ -12733,43 +12733,43 @@
         <v/>
       </c>
       <c r="E17" s="55">
-        <f>MRP!E94</f>
+        <f>IF($A17="","",MRP!E94)</f>
         <v/>
       </c>
       <c r="F17" s="55">
-        <f>MRP!F94</f>
+        <f>IF($A17="","",MRP!F94)</f>
         <v/>
       </c>
       <c r="G17" s="55">
-        <f>MRP!G94</f>
+        <f>IF($A17="","",MRP!G94)</f>
         <v/>
       </c>
       <c r="H17" s="55">
-        <f>MRP!H94</f>
+        <f>IF($A17="","",MRP!H94)</f>
         <v/>
       </c>
       <c r="I17" s="55">
-        <f>MRP!I94</f>
+        <f>IF($A17="","",MRP!I94)</f>
         <v/>
       </c>
       <c r="J17" s="55">
-        <f>MRP!J94</f>
+        <f>IF($A17="","",MRP!J94)</f>
         <v/>
       </c>
       <c r="K17" s="55">
-        <f>MRP!K94</f>
+        <f>IF($A17="","",MRP!K94)</f>
         <v/>
       </c>
       <c r="L17" s="55">
-        <f>MRP!L94</f>
+        <f>IF($A17="","",MRP!L94)</f>
         <v/>
       </c>
       <c r="M17" s="56">
-        <f>SUM(E17:L17)</f>
+        <f>IF($A17="","",SUM(E17:L17))</f>
         <v/>
       </c>
       <c r="N17" s="57">
-        <f>M17*D17</f>
+        <f>IF($A17="","",M17*D17)</f>
         <v/>
       </c>
     </row>
@@ -12791,43 +12791,43 @@
         <v/>
       </c>
       <c r="E18" s="55">
-        <f>MRP!E101</f>
+        <f>IF($A18="","",MRP!E101)</f>
         <v/>
       </c>
       <c r="F18" s="55">
-        <f>MRP!F101</f>
+        <f>IF($A18="","",MRP!F101)</f>
         <v/>
       </c>
       <c r="G18" s="55">
-        <f>MRP!G101</f>
+        <f>IF($A18="","",MRP!G101)</f>
         <v/>
       </c>
       <c r="H18" s="55">
-        <f>MRP!H101</f>
+        <f>IF($A18="","",MRP!H101)</f>
         <v/>
       </c>
       <c r="I18" s="55">
-        <f>MRP!I101</f>
+        <f>IF($A18="","",MRP!I101)</f>
         <v/>
       </c>
       <c r="J18" s="55">
-        <f>MRP!J101</f>
+        <f>IF($A18="","",MRP!J101)</f>
         <v/>
       </c>
       <c r="K18" s="55">
-        <f>MRP!K101</f>
+        <f>IF($A18="","",MRP!K101)</f>
         <v/>
       </c>
       <c r="L18" s="55">
-        <f>MRP!L101</f>
+        <f>IF($A18="","",MRP!L101)</f>
         <v/>
       </c>
       <c r="M18" s="56">
-        <f>SUM(E18:L18)</f>
+        <f>IF($A18="","",SUM(E18:L18))</f>
         <v/>
       </c>
       <c r="N18" s="57">
-        <f>M18*D18</f>
+        <f>IF($A18="","",M18*D18)</f>
         <v/>
       </c>
     </row>
@@ -12849,43 +12849,43 @@
         <v/>
       </c>
       <c r="E19" s="55">
-        <f>MRP!E108</f>
+        <f>IF($A19="","",MRP!E108)</f>
         <v/>
       </c>
       <c r="F19" s="55">
-        <f>MRP!F108</f>
+        <f>IF($A19="","",MRP!F108)</f>
         <v/>
       </c>
       <c r="G19" s="55">
-        <f>MRP!G108</f>
+        <f>IF($A19="","",MRP!G108)</f>
         <v/>
       </c>
       <c r="H19" s="55">
-        <f>MRP!H108</f>
+        <f>IF($A19="","",MRP!H108)</f>
         <v/>
       </c>
       <c r="I19" s="55">
-        <f>MRP!I108</f>
+        <f>IF($A19="","",MRP!I108)</f>
         <v/>
       </c>
       <c r="J19" s="55">
-        <f>MRP!J108</f>
+        <f>IF($A19="","",MRP!J108)</f>
         <v/>
       </c>
       <c r="K19" s="55">
-        <f>MRP!K108</f>
+        <f>IF($A19="","",MRP!K108)</f>
         <v/>
       </c>
       <c r="L19" s="55">
-        <f>MRP!L108</f>
+        <f>IF($A19="","",MRP!L108)</f>
         <v/>
       </c>
       <c r="M19" s="56">
-        <f>SUM(E19:L19)</f>
+        <f>IF($A19="","",SUM(E19:L19))</f>
         <v/>
       </c>
       <c r="N19" s="57">
-        <f>M19*D19</f>
+        <f>IF($A19="","",M19*D19)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar corrida MRP de ejemplo de un mes y blindar el redondeo del lote
Corrida (MRP_ATMIN_corrida_ejemplo_mes.xlsx): mes de setiembre 2026 con
los estandares de sostenimiento reales de RA Brenda (1 cimbra por disparo
de 1.5 m) y CRNE (1 malla + 11 pernos por disparo de 1.5 m, seccion
3.5x3.5). Incluye hoja RESUMEN MES con la conversion del estandar, el plan
de avance, el consumo del mes y las ordenes a lanzar.

Plantilla: la necesidad bruta y la necesidad neta ahora se redondean a 4
decimales antes del ROUNDUP al lote de compra. Sin eso, un estandar
capturado con decimales truncados (0.666667) generaba un sobrante de 4e-6
que empujaba el redondeo un lote completo hacia arriba: pedia 15 cimbras
donde correspondian 10.

Verificado con evaluacion de todas las formulas: 0 celdas con error y las
15 filas del calculo coinciden con el desarrollo hecho a mano.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KofGASuDqP2DkSsvGxsHDK
</commit_message>
<xml_diff>
--- a/MRP_ATMIN_plantilla.xlsx
+++ b/MRP_ATMIN_plantilla.xlsx
@@ -7575,35 +7575,35 @@
       </c>
       <c r="D5" s="44" t="n"/>
       <c r="E5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L5" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A5,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M5" s="46" t="n"/>
@@ -7701,35 +7701,35 @@
       </c>
       <c r="D8" s="44" t="n"/>
       <c r="E8" s="49">
-        <f>MAX(0,E5+Materiales!$H$4-D7-E6)</f>
+        <f>MAX(0,ROUND(E5+Materiales!$H$4-D7-E6,4))</f>
         <v/>
       </c>
       <c r="F8" s="49">
-        <f>MAX(0,F5+Materiales!$H$4-E7-F6)</f>
+        <f>MAX(0,ROUND(F5+Materiales!$H$4-E7-F6,4))</f>
         <v/>
       </c>
       <c r="G8" s="49">
-        <f>MAX(0,G5+Materiales!$H$4-F7-G6)</f>
+        <f>MAX(0,ROUND(G5+Materiales!$H$4-F7-G6,4))</f>
         <v/>
       </c>
       <c r="H8" s="49">
-        <f>MAX(0,H5+Materiales!$H$4-G7-H6)</f>
+        <f>MAX(0,ROUND(H5+Materiales!$H$4-G7-H6,4))</f>
         <v/>
       </c>
       <c r="I8" s="49">
-        <f>MAX(0,I5+Materiales!$H$4-H7-I6)</f>
+        <f>MAX(0,ROUND(I5+Materiales!$H$4-H7-I6,4))</f>
         <v/>
       </c>
       <c r="J8" s="49">
-        <f>MAX(0,J5+Materiales!$H$4-I7-J6)</f>
+        <f>MAX(0,ROUND(J5+Materiales!$H$4-I7-J6,4))</f>
         <v/>
       </c>
       <c r="K8" s="49">
-        <f>MAX(0,K5+Materiales!$H$4-J7-K6)</f>
+        <f>MAX(0,ROUND(K5+Materiales!$H$4-J7-K6,4))</f>
         <v/>
       </c>
       <c r="L8" s="49">
-        <f>MAX(0,L5+Materiales!$H$4-K7-L6)</f>
+        <f>MAX(0,ROUND(L5+Materiales!$H$4-K7-L6,4))</f>
         <v/>
       </c>
       <c r="M8" s="46" t="n"/>
@@ -7850,35 +7850,35 @@
       </c>
       <c r="D12" s="44" t="n"/>
       <c r="E12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L12" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A12,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M12" s="46" t="n"/>
@@ -7976,35 +7976,35 @@
       </c>
       <c r="D15" s="44" t="n"/>
       <c r="E15" s="49">
-        <f>MAX(0,E12+Materiales!$H$5-D14-E13)</f>
+        <f>MAX(0,ROUND(E12+Materiales!$H$5-D14-E13,4))</f>
         <v/>
       </c>
       <c r="F15" s="49">
-        <f>MAX(0,F12+Materiales!$H$5-E14-F13)</f>
+        <f>MAX(0,ROUND(F12+Materiales!$H$5-E14-F13,4))</f>
         <v/>
       </c>
       <c r="G15" s="49">
-        <f>MAX(0,G12+Materiales!$H$5-F14-G13)</f>
+        <f>MAX(0,ROUND(G12+Materiales!$H$5-F14-G13,4))</f>
         <v/>
       </c>
       <c r="H15" s="49">
-        <f>MAX(0,H12+Materiales!$H$5-G14-H13)</f>
+        <f>MAX(0,ROUND(H12+Materiales!$H$5-G14-H13,4))</f>
         <v/>
       </c>
       <c r="I15" s="49">
-        <f>MAX(0,I12+Materiales!$H$5-H14-I13)</f>
+        <f>MAX(0,ROUND(I12+Materiales!$H$5-H14-I13,4))</f>
         <v/>
       </c>
       <c r="J15" s="49">
-        <f>MAX(0,J12+Materiales!$H$5-I14-J13)</f>
+        <f>MAX(0,ROUND(J12+Materiales!$H$5-I14-J13,4))</f>
         <v/>
       </c>
       <c r="K15" s="49">
-        <f>MAX(0,K12+Materiales!$H$5-J14-K13)</f>
+        <f>MAX(0,ROUND(K12+Materiales!$H$5-J14-K13,4))</f>
         <v/>
       </c>
       <c r="L15" s="49">
-        <f>MAX(0,L12+Materiales!$H$5-K14-L13)</f>
+        <f>MAX(0,ROUND(L12+Materiales!$H$5-K14-L13,4))</f>
         <v/>
       </c>
       <c r="M15" s="46" t="n"/>
@@ -8125,35 +8125,35 @@
       </c>
       <c r="D19" s="44" t="n"/>
       <c r="E19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L19" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A19,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M19" s="46" t="n"/>
@@ -8251,35 +8251,35 @@
       </c>
       <c r="D22" s="44" t="n"/>
       <c r="E22" s="49">
-        <f>MAX(0,E19+Materiales!$H$6-D21-E20)</f>
+        <f>MAX(0,ROUND(E19+Materiales!$H$6-D21-E20,4))</f>
         <v/>
       </c>
       <c r="F22" s="49">
-        <f>MAX(0,F19+Materiales!$H$6-E21-F20)</f>
+        <f>MAX(0,ROUND(F19+Materiales!$H$6-E21-F20,4))</f>
         <v/>
       </c>
       <c r="G22" s="49">
-        <f>MAX(0,G19+Materiales!$H$6-F21-G20)</f>
+        <f>MAX(0,ROUND(G19+Materiales!$H$6-F21-G20,4))</f>
         <v/>
       </c>
       <c r="H22" s="49">
-        <f>MAX(0,H19+Materiales!$H$6-G21-H20)</f>
+        <f>MAX(0,ROUND(H19+Materiales!$H$6-G21-H20,4))</f>
         <v/>
       </c>
       <c r="I22" s="49">
-        <f>MAX(0,I19+Materiales!$H$6-H21-I20)</f>
+        <f>MAX(0,ROUND(I19+Materiales!$H$6-H21-I20,4))</f>
         <v/>
       </c>
       <c r="J22" s="49">
-        <f>MAX(0,J19+Materiales!$H$6-I21-J20)</f>
+        <f>MAX(0,ROUND(J19+Materiales!$H$6-I21-J20,4))</f>
         <v/>
       </c>
       <c r="K22" s="49">
-        <f>MAX(0,K19+Materiales!$H$6-J21-K20)</f>
+        <f>MAX(0,ROUND(K19+Materiales!$H$6-J21-K20,4))</f>
         <v/>
       </c>
       <c r="L22" s="49">
-        <f>MAX(0,L19+Materiales!$H$6-K21-L20)</f>
+        <f>MAX(0,ROUND(L19+Materiales!$H$6-K21-L20,4))</f>
         <v/>
       </c>
       <c r="M22" s="46" t="n"/>
@@ -8400,35 +8400,35 @@
       </c>
       <c r="D26" s="44" t="n"/>
       <c r="E26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L26" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A26,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M26" s="46" t="n"/>
@@ -8526,35 +8526,35 @@
       </c>
       <c r="D29" s="44" t="n"/>
       <c r="E29" s="49">
-        <f>MAX(0,E26+Materiales!$H$7-D28-E27)</f>
+        <f>MAX(0,ROUND(E26+Materiales!$H$7-D28-E27,4))</f>
         <v/>
       </c>
       <c r="F29" s="49">
-        <f>MAX(0,F26+Materiales!$H$7-E28-F27)</f>
+        <f>MAX(0,ROUND(F26+Materiales!$H$7-E28-F27,4))</f>
         <v/>
       </c>
       <c r="G29" s="49">
-        <f>MAX(0,G26+Materiales!$H$7-F28-G27)</f>
+        <f>MAX(0,ROUND(G26+Materiales!$H$7-F28-G27,4))</f>
         <v/>
       </c>
       <c r="H29" s="49">
-        <f>MAX(0,H26+Materiales!$H$7-G28-H27)</f>
+        <f>MAX(0,ROUND(H26+Materiales!$H$7-G28-H27,4))</f>
         <v/>
       </c>
       <c r="I29" s="49">
-        <f>MAX(0,I26+Materiales!$H$7-H28-I27)</f>
+        <f>MAX(0,ROUND(I26+Materiales!$H$7-H28-I27,4))</f>
         <v/>
       </c>
       <c r="J29" s="49">
-        <f>MAX(0,J26+Materiales!$H$7-I28-J27)</f>
+        <f>MAX(0,ROUND(J26+Materiales!$H$7-I28-J27,4))</f>
         <v/>
       </c>
       <c r="K29" s="49">
-        <f>MAX(0,K26+Materiales!$H$7-J28-K27)</f>
+        <f>MAX(0,ROUND(K26+Materiales!$H$7-J28-K27,4))</f>
         <v/>
       </c>
       <c r="L29" s="49">
-        <f>MAX(0,L26+Materiales!$H$7-K28-L27)</f>
+        <f>MAX(0,ROUND(L26+Materiales!$H$7-K28-L27,4))</f>
         <v/>
       </c>
       <c r="M29" s="46" t="n"/>
@@ -8675,35 +8675,35 @@
       </c>
       <c r="D33" s="44" t="n"/>
       <c r="E33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L33" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A33,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M33" s="46" t="n"/>
@@ -8801,35 +8801,35 @@
       </c>
       <c r="D36" s="44" t="n"/>
       <c r="E36" s="49">
-        <f>MAX(0,E33+Materiales!$H$8-D35-E34)</f>
+        <f>MAX(0,ROUND(E33+Materiales!$H$8-D35-E34,4))</f>
         <v/>
       </c>
       <c r="F36" s="49">
-        <f>MAX(0,F33+Materiales!$H$8-E35-F34)</f>
+        <f>MAX(0,ROUND(F33+Materiales!$H$8-E35-F34,4))</f>
         <v/>
       </c>
       <c r="G36" s="49">
-        <f>MAX(0,G33+Materiales!$H$8-F35-G34)</f>
+        <f>MAX(0,ROUND(G33+Materiales!$H$8-F35-G34,4))</f>
         <v/>
       </c>
       <c r="H36" s="49">
-        <f>MAX(0,H33+Materiales!$H$8-G35-H34)</f>
+        <f>MAX(0,ROUND(H33+Materiales!$H$8-G35-H34,4))</f>
         <v/>
       </c>
       <c r="I36" s="49">
-        <f>MAX(0,I33+Materiales!$H$8-H35-I34)</f>
+        <f>MAX(0,ROUND(I33+Materiales!$H$8-H35-I34,4))</f>
         <v/>
       </c>
       <c r="J36" s="49">
-        <f>MAX(0,J33+Materiales!$H$8-I35-J34)</f>
+        <f>MAX(0,ROUND(J33+Materiales!$H$8-I35-J34,4))</f>
         <v/>
       </c>
       <c r="K36" s="49">
-        <f>MAX(0,K33+Materiales!$H$8-J35-K34)</f>
+        <f>MAX(0,ROUND(K33+Materiales!$H$8-J35-K34,4))</f>
         <v/>
       </c>
       <c r="L36" s="49">
-        <f>MAX(0,L33+Materiales!$H$8-K35-L34)</f>
+        <f>MAX(0,ROUND(L33+Materiales!$H$8-K35-L34,4))</f>
         <v/>
       </c>
       <c r="M36" s="46" t="n"/>
@@ -8950,35 +8950,35 @@
       </c>
       <c r="D40" s="44" t="n"/>
       <c r="E40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L40" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A40,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M40" s="46" t="n"/>
@@ -9076,35 +9076,35 @@
       </c>
       <c r="D43" s="44" t="n"/>
       <c r="E43" s="49">
-        <f>MAX(0,E40+Materiales!$H$9-D42-E41)</f>
+        <f>MAX(0,ROUND(E40+Materiales!$H$9-D42-E41,4))</f>
         <v/>
       </c>
       <c r="F43" s="49">
-        <f>MAX(0,F40+Materiales!$H$9-E42-F41)</f>
+        <f>MAX(0,ROUND(F40+Materiales!$H$9-E42-F41,4))</f>
         <v/>
       </c>
       <c r="G43" s="49">
-        <f>MAX(0,G40+Materiales!$H$9-F42-G41)</f>
+        <f>MAX(0,ROUND(G40+Materiales!$H$9-F42-G41,4))</f>
         <v/>
       </c>
       <c r="H43" s="49">
-        <f>MAX(0,H40+Materiales!$H$9-G42-H41)</f>
+        <f>MAX(0,ROUND(H40+Materiales!$H$9-G42-H41,4))</f>
         <v/>
       </c>
       <c r="I43" s="49">
-        <f>MAX(0,I40+Materiales!$H$9-H42-I41)</f>
+        <f>MAX(0,ROUND(I40+Materiales!$H$9-H42-I41,4))</f>
         <v/>
       </c>
       <c r="J43" s="49">
-        <f>MAX(0,J40+Materiales!$H$9-I42-J41)</f>
+        <f>MAX(0,ROUND(J40+Materiales!$H$9-I42-J41,4))</f>
         <v/>
       </c>
       <c r="K43" s="49">
-        <f>MAX(0,K40+Materiales!$H$9-J42-K41)</f>
+        <f>MAX(0,ROUND(K40+Materiales!$H$9-J42-K41,4))</f>
         <v/>
       </c>
       <c r="L43" s="49">
-        <f>MAX(0,L40+Materiales!$H$9-K42-L41)</f>
+        <f>MAX(0,ROUND(L40+Materiales!$H$9-K42-L41,4))</f>
         <v/>
       </c>
       <c r="M43" s="46" t="n"/>
@@ -9225,35 +9225,35 @@
       </c>
       <c r="D47" s="44" t="n"/>
       <c r="E47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L47" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A47,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M47" s="46" t="n"/>
@@ -9351,35 +9351,35 @@
       </c>
       <c r="D50" s="44" t="n"/>
       <c r="E50" s="49">
-        <f>MAX(0,E47+Materiales!$H$10-D49-E48)</f>
+        <f>MAX(0,ROUND(E47+Materiales!$H$10-D49-E48,4))</f>
         <v/>
       </c>
       <c r="F50" s="49">
-        <f>MAX(0,F47+Materiales!$H$10-E49-F48)</f>
+        <f>MAX(0,ROUND(F47+Materiales!$H$10-E49-F48,4))</f>
         <v/>
       </c>
       <c r="G50" s="49">
-        <f>MAX(0,G47+Materiales!$H$10-F49-G48)</f>
+        <f>MAX(0,ROUND(G47+Materiales!$H$10-F49-G48,4))</f>
         <v/>
       </c>
       <c r="H50" s="49">
-        <f>MAX(0,H47+Materiales!$H$10-G49-H48)</f>
+        <f>MAX(0,ROUND(H47+Materiales!$H$10-G49-H48,4))</f>
         <v/>
       </c>
       <c r="I50" s="49">
-        <f>MAX(0,I47+Materiales!$H$10-H49-I48)</f>
+        <f>MAX(0,ROUND(I47+Materiales!$H$10-H49-I48,4))</f>
         <v/>
       </c>
       <c r="J50" s="49">
-        <f>MAX(0,J47+Materiales!$H$10-I49-J48)</f>
+        <f>MAX(0,ROUND(J47+Materiales!$H$10-I49-J48,4))</f>
         <v/>
       </c>
       <c r="K50" s="49">
-        <f>MAX(0,K47+Materiales!$H$10-J49-K48)</f>
+        <f>MAX(0,ROUND(K47+Materiales!$H$10-J49-K48,4))</f>
         <v/>
       </c>
       <c r="L50" s="49">
-        <f>MAX(0,L47+Materiales!$H$10-K49-L48)</f>
+        <f>MAX(0,ROUND(L47+Materiales!$H$10-K49-L48,4))</f>
         <v/>
       </c>
       <c r="M50" s="46" t="n"/>
@@ -9500,35 +9500,35 @@
       </c>
       <c r="D54" s="44" t="n"/>
       <c r="E54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L54" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A54,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M54" s="46" t="n"/>
@@ -9626,35 +9626,35 @@
       </c>
       <c r="D57" s="44" t="n"/>
       <c r="E57" s="49">
-        <f>MAX(0,E54+Materiales!$H$11-D56-E55)</f>
+        <f>MAX(0,ROUND(E54+Materiales!$H$11-D56-E55,4))</f>
         <v/>
       </c>
       <c r="F57" s="49">
-        <f>MAX(0,F54+Materiales!$H$11-E56-F55)</f>
+        <f>MAX(0,ROUND(F54+Materiales!$H$11-E56-F55,4))</f>
         <v/>
       </c>
       <c r="G57" s="49">
-        <f>MAX(0,G54+Materiales!$H$11-F56-G55)</f>
+        <f>MAX(0,ROUND(G54+Materiales!$H$11-F56-G55,4))</f>
         <v/>
       </c>
       <c r="H57" s="49">
-        <f>MAX(0,H54+Materiales!$H$11-G56-H55)</f>
+        <f>MAX(0,ROUND(H54+Materiales!$H$11-G56-H55,4))</f>
         <v/>
       </c>
       <c r="I57" s="49">
-        <f>MAX(0,I54+Materiales!$H$11-H56-I55)</f>
+        <f>MAX(0,ROUND(I54+Materiales!$H$11-H56-I55,4))</f>
         <v/>
       </c>
       <c r="J57" s="49">
-        <f>MAX(0,J54+Materiales!$H$11-I56-J55)</f>
+        <f>MAX(0,ROUND(J54+Materiales!$H$11-I56-J55,4))</f>
         <v/>
       </c>
       <c r="K57" s="49">
-        <f>MAX(0,K54+Materiales!$H$11-J56-K55)</f>
+        <f>MAX(0,ROUND(K54+Materiales!$H$11-J56-K55,4))</f>
         <v/>
       </c>
       <c r="L57" s="49">
-        <f>MAX(0,L54+Materiales!$H$11-K56-L55)</f>
+        <f>MAX(0,ROUND(L54+Materiales!$H$11-K56-L55,4))</f>
         <v/>
       </c>
       <c r="M57" s="46" t="n"/>
@@ -9775,35 +9775,35 @@
       </c>
       <c r="D61" s="44" t="n"/>
       <c r="E61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L61" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A61,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M61" s="46" t="n"/>
@@ -9901,35 +9901,35 @@
       </c>
       <c r="D64" s="44" t="n"/>
       <c r="E64" s="49">
-        <f>MAX(0,E61+Materiales!$H$12-D63-E62)</f>
+        <f>MAX(0,ROUND(E61+Materiales!$H$12-D63-E62,4))</f>
         <v/>
       </c>
       <c r="F64" s="49">
-        <f>MAX(0,F61+Materiales!$H$12-E63-F62)</f>
+        <f>MAX(0,ROUND(F61+Materiales!$H$12-E63-F62,4))</f>
         <v/>
       </c>
       <c r="G64" s="49">
-        <f>MAX(0,G61+Materiales!$H$12-F63-G62)</f>
+        <f>MAX(0,ROUND(G61+Materiales!$H$12-F63-G62,4))</f>
         <v/>
       </c>
       <c r="H64" s="49">
-        <f>MAX(0,H61+Materiales!$H$12-G63-H62)</f>
+        <f>MAX(0,ROUND(H61+Materiales!$H$12-G63-H62,4))</f>
         <v/>
       </c>
       <c r="I64" s="49">
-        <f>MAX(0,I61+Materiales!$H$12-H63-I62)</f>
+        <f>MAX(0,ROUND(I61+Materiales!$H$12-H63-I62,4))</f>
         <v/>
       </c>
       <c r="J64" s="49">
-        <f>MAX(0,J61+Materiales!$H$12-I63-J62)</f>
+        <f>MAX(0,ROUND(J61+Materiales!$H$12-I63-J62,4))</f>
         <v/>
       </c>
       <c r="K64" s="49">
-        <f>MAX(0,K61+Materiales!$H$12-J63-K62)</f>
+        <f>MAX(0,ROUND(K61+Materiales!$H$12-J63-K62,4))</f>
         <v/>
       </c>
       <c r="L64" s="49">
-        <f>MAX(0,L61+Materiales!$H$12-K63-L62)</f>
+        <f>MAX(0,ROUND(L61+Materiales!$H$12-K63-L62,4))</f>
         <v/>
       </c>
       <c r="M64" s="46" t="n"/>
@@ -10050,35 +10050,35 @@
       </c>
       <c r="D68" s="44" t="n"/>
       <c r="E68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L68" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A68,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M68" s="46" t="n"/>
@@ -10176,35 +10176,35 @@
       </c>
       <c r="D71" s="44" t="n"/>
       <c r="E71" s="49">
-        <f>MAX(0,E68+Materiales!$H$13-D70-E69)</f>
+        <f>MAX(0,ROUND(E68+Materiales!$H$13-D70-E69,4))</f>
         <v/>
       </c>
       <c r="F71" s="49">
-        <f>MAX(0,F68+Materiales!$H$13-E70-F69)</f>
+        <f>MAX(0,ROUND(F68+Materiales!$H$13-E70-F69,4))</f>
         <v/>
       </c>
       <c r="G71" s="49">
-        <f>MAX(0,G68+Materiales!$H$13-F70-G69)</f>
+        <f>MAX(0,ROUND(G68+Materiales!$H$13-F70-G69,4))</f>
         <v/>
       </c>
       <c r="H71" s="49">
-        <f>MAX(0,H68+Materiales!$H$13-G70-H69)</f>
+        <f>MAX(0,ROUND(H68+Materiales!$H$13-G70-H69,4))</f>
         <v/>
       </c>
       <c r="I71" s="49">
-        <f>MAX(0,I68+Materiales!$H$13-H70-I69)</f>
+        <f>MAX(0,ROUND(I68+Materiales!$H$13-H70-I69,4))</f>
         <v/>
       </c>
       <c r="J71" s="49">
-        <f>MAX(0,J68+Materiales!$H$13-I70-J69)</f>
+        <f>MAX(0,ROUND(J68+Materiales!$H$13-I70-J69,4))</f>
         <v/>
       </c>
       <c r="K71" s="49">
-        <f>MAX(0,K68+Materiales!$H$13-J70-K69)</f>
+        <f>MAX(0,ROUND(K68+Materiales!$H$13-J70-K69,4))</f>
         <v/>
       </c>
       <c r="L71" s="49">
-        <f>MAX(0,L68+Materiales!$H$13-K70-L69)</f>
+        <f>MAX(0,ROUND(L68+Materiales!$H$13-K70-L69,4))</f>
         <v/>
       </c>
       <c r="M71" s="46" t="n"/>
@@ -10325,35 +10325,35 @@
       </c>
       <c r="D75" s="44" t="n"/>
       <c r="E75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L75" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A75,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M75" s="46" t="n"/>
@@ -10451,35 +10451,35 @@
       </c>
       <c r="D78" s="44" t="n"/>
       <c r="E78" s="49">
-        <f>MAX(0,E75+Materiales!$H$14-D77-E76)</f>
+        <f>MAX(0,ROUND(E75+Materiales!$H$14-D77-E76,4))</f>
         <v/>
       </c>
       <c r="F78" s="49">
-        <f>MAX(0,F75+Materiales!$H$14-E77-F76)</f>
+        <f>MAX(0,ROUND(F75+Materiales!$H$14-E77-F76,4))</f>
         <v/>
       </c>
       <c r="G78" s="49">
-        <f>MAX(0,G75+Materiales!$H$14-F77-G76)</f>
+        <f>MAX(0,ROUND(G75+Materiales!$H$14-F77-G76,4))</f>
         <v/>
       </c>
       <c r="H78" s="49">
-        <f>MAX(0,H75+Materiales!$H$14-G77-H76)</f>
+        <f>MAX(0,ROUND(H75+Materiales!$H$14-G77-H76,4))</f>
         <v/>
       </c>
       <c r="I78" s="49">
-        <f>MAX(0,I75+Materiales!$H$14-H77-I76)</f>
+        <f>MAX(0,ROUND(I75+Materiales!$H$14-H77-I76,4))</f>
         <v/>
       </c>
       <c r="J78" s="49">
-        <f>MAX(0,J75+Materiales!$H$14-I77-J76)</f>
+        <f>MAX(0,ROUND(J75+Materiales!$H$14-I77-J76,4))</f>
         <v/>
       </c>
       <c r="K78" s="49">
-        <f>MAX(0,K75+Materiales!$H$14-J77-K76)</f>
+        <f>MAX(0,ROUND(K75+Materiales!$H$14-J77-K76,4))</f>
         <v/>
       </c>
       <c r="L78" s="49">
-        <f>MAX(0,L75+Materiales!$H$14-K77-L76)</f>
+        <f>MAX(0,ROUND(L75+Materiales!$H$14-K77-L76,4))</f>
         <v/>
       </c>
       <c r="M78" s="46" t="n"/>
@@ -10600,35 +10600,35 @@
       </c>
       <c r="D82" s="44" t="n"/>
       <c r="E82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L82" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A82,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M82" s="46" t="n"/>
@@ -10726,35 +10726,35 @@
       </c>
       <c r="D85" s="44" t="n"/>
       <c r="E85" s="49">
-        <f>MAX(0,E82+Materiales!$H$15-D84-E83)</f>
+        <f>MAX(0,ROUND(E82+Materiales!$H$15-D84-E83,4))</f>
         <v/>
       </c>
       <c r="F85" s="49">
-        <f>MAX(0,F82+Materiales!$H$15-E84-F83)</f>
+        <f>MAX(0,ROUND(F82+Materiales!$H$15-E84-F83,4))</f>
         <v/>
       </c>
       <c r="G85" s="49">
-        <f>MAX(0,G82+Materiales!$H$15-F84-G83)</f>
+        <f>MAX(0,ROUND(G82+Materiales!$H$15-F84-G83,4))</f>
         <v/>
       </c>
       <c r="H85" s="49">
-        <f>MAX(0,H82+Materiales!$H$15-G84-H83)</f>
+        <f>MAX(0,ROUND(H82+Materiales!$H$15-G84-H83,4))</f>
         <v/>
       </c>
       <c r="I85" s="49">
-        <f>MAX(0,I82+Materiales!$H$15-H84-I83)</f>
+        <f>MAX(0,ROUND(I82+Materiales!$H$15-H84-I83,4))</f>
         <v/>
       </c>
       <c r="J85" s="49">
-        <f>MAX(0,J82+Materiales!$H$15-I84-J83)</f>
+        <f>MAX(0,ROUND(J82+Materiales!$H$15-I84-J83,4))</f>
         <v/>
       </c>
       <c r="K85" s="49">
-        <f>MAX(0,K82+Materiales!$H$15-J84-K83)</f>
+        <f>MAX(0,ROUND(K82+Materiales!$H$15-J84-K83,4))</f>
         <v/>
       </c>
       <c r="L85" s="49">
-        <f>MAX(0,L82+Materiales!$H$15-K84-L83)</f>
+        <f>MAX(0,ROUND(L82+Materiales!$H$15-K84-L83,4))</f>
         <v/>
       </c>
       <c r="M85" s="46" t="n"/>
@@ -10875,35 +10875,35 @@
       </c>
       <c r="D89" s="44" t="n"/>
       <c r="E89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L89" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A89,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M89" s="46" t="n"/>
@@ -11001,35 +11001,35 @@
       </c>
       <c r="D92" s="44" t="n"/>
       <c r="E92" s="49">
-        <f>MAX(0,E89+Materiales!$H$16-D91-E90)</f>
+        <f>MAX(0,ROUND(E89+Materiales!$H$16-D91-E90,4))</f>
         <v/>
       </c>
       <c r="F92" s="49">
-        <f>MAX(0,F89+Materiales!$H$16-E91-F90)</f>
+        <f>MAX(0,ROUND(F89+Materiales!$H$16-E91-F90,4))</f>
         <v/>
       </c>
       <c r="G92" s="49">
-        <f>MAX(0,G89+Materiales!$H$16-F91-G90)</f>
+        <f>MAX(0,ROUND(G89+Materiales!$H$16-F91-G90,4))</f>
         <v/>
       </c>
       <c r="H92" s="49">
-        <f>MAX(0,H89+Materiales!$H$16-G91-H90)</f>
+        <f>MAX(0,ROUND(H89+Materiales!$H$16-G91-H90,4))</f>
         <v/>
       </c>
       <c r="I92" s="49">
-        <f>MAX(0,I89+Materiales!$H$16-H91-I90)</f>
+        <f>MAX(0,ROUND(I89+Materiales!$H$16-H91-I90,4))</f>
         <v/>
       </c>
       <c r="J92" s="49">
-        <f>MAX(0,J89+Materiales!$H$16-I91-J90)</f>
+        <f>MAX(0,ROUND(J89+Materiales!$H$16-I91-J90,4))</f>
         <v/>
       </c>
       <c r="K92" s="49">
-        <f>MAX(0,K89+Materiales!$H$16-J91-K90)</f>
+        <f>MAX(0,ROUND(K89+Materiales!$H$16-J91-K90,4))</f>
         <v/>
       </c>
       <c r="L92" s="49">
-        <f>MAX(0,L89+Materiales!$H$16-K91-L90)</f>
+        <f>MAX(0,ROUND(L89+Materiales!$H$16-K91-L90,4))</f>
         <v/>
       </c>
       <c r="M92" s="46" t="n"/>
@@ -11150,35 +11150,35 @@
       </c>
       <c r="D96" s="44" t="n"/>
       <c r="E96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L96" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A96,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M96" s="46" t="n"/>
@@ -11276,35 +11276,35 @@
       </c>
       <c r="D99" s="44" t="n"/>
       <c r="E99" s="49">
-        <f>MAX(0,E96+Materiales!$H$17-D98-E97)</f>
+        <f>MAX(0,ROUND(E96+Materiales!$H$17-D98-E97,4))</f>
         <v/>
       </c>
       <c r="F99" s="49">
-        <f>MAX(0,F96+Materiales!$H$17-E98-F97)</f>
+        <f>MAX(0,ROUND(F96+Materiales!$H$17-E98-F97,4))</f>
         <v/>
       </c>
       <c r="G99" s="49">
-        <f>MAX(0,G96+Materiales!$H$17-F98-G97)</f>
+        <f>MAX(0,ROUND(G96+Materiales!$H$17-F98-G97,4))</f>
         <v/>
       </c>
       <c r="H99" s="49">
-        <f>MAX(0,H96+Materiales!$H$17-G98-H97)</f>
+        <f>MAX(0,ROUND(H96+Materiales!$H$17-G98-H97,4))</f>
         <v/>
       </c>
       <c r="I99" s="49">
-        <f>MAX(0,I96+Materiales!$H$17-H98-I97)</f>
+        <f>MAX(0,ROUND(I96+Materiales!$H$17-H98-I97,4))</f>
         <v/>
       </c>
       <c r="J99" s="49">
-        <f>MAX(0,J96+Materiales!$H$17-I98-J97)</f>
+        <f>MAX(0,ROUND(J96+Materiales!$H$17-I98-J97,4))</f>
         <v/>
       </c>
       <c r="K99" s="49">
-        <f>MAX(0,K96+Materiales!$H$17-J98-K97)</f>
+        <f>MAX(0,ROUND(K96+Materiales!$H$17-J98-K97,4))</f>
         <v/>
       </c>
       <c r="L99" s="49">
-        <f>MAX(0,L96+Materiales!$H$17-K98-L97)</f>
+        <f>MAX(0,ROUND(L96+Materiales!$H$17-K98-L97,4))</f>
         <v/>
       </c>
       <c r="M99" s="46" t="n"/>
@@ -11425,35 +11425,35 @@
       </c>
       <c r="D103" s="44" t="n"/>
       <c r="E103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!G$4:G$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!G$4:G$103),4)</f>
         <v/>
       </c>
       <c r="F103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!H$4:H$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!H$4:H$103),4)</f>
         <v/>
       </c>
       <c r="G103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!I$4:I$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!I$4:I$103),4)</f>
         <v/>
       </c>
       <c r="H103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!J$4:J$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!J$4:J$103),4)</f>
         <v/>
       </c>
       <c r="I103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!K$4:K$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!K$4:K$103),4)</f>
         <v/>
       </c>
       <c r="J103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!L$4:L$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!L$4:L$103),4)</f>
         <v/>
       </c>
       <c r="K103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!M$4:M$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!M$4:M$103),4)</f>
         <v/>
       </c>
       <c r="L103" s="45">
-        <f>SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!N$4:N$103)</f>
+        <f>ROUND(SUMIF(Consumo!$B$4:$B$103,$A103,Consumo!N$4:N$103),4)</f>
         <v/>
       </c>
       <c r="M103" s="46" t="n"/>
@@ -11551,35 +11551,35 @@
       </c>
       <c r="D106" s="44" t="n"/>
       <c r="E106" s="49">
-        <f>MAX(0,E103+Materiales!$H$18-D105-E104)</f>
+        <f>MAX(0,ROUND(E103+Materiales!$H$18-D105-E104,4))</f>
         <v/>
       </c>
       <c r="F106" s="49">
-        <f>MAX(0,F103+Materiales!$H$18-E105-F104)</f>
+        <f>MAX(0,ROUND(F103+Materiales!$H$18-E105-F104,4))</f>
         <v/>
       </c>
       <c r="G106" s="49">
-        <f>MAX(0,G103+Materiales!$H$18-F105-G104)</f>
+        <f>MAX(0,ROUND(G103+Materiales!$H$18-F105-G104,4))</f>
         <v/>
       </c>
       <c r="H106" s="49">
-        <f>MAX(0,H103+Materiales!$H$18-G105-H104)</f>
+        <f>MAX(0,ROUND(H103+Materiales!$H$18-G105-H104,4))</f>
         <v/>
       </c>
       <c r="I106" s="49">
-        <f>MAX(0,I103+Materiales!$H$18-H105-I104)</f>
+        <f>MAX(0,ROUND(I103+Materiales!$H$18-H105-I104,4))</f>
         <v/>
       </c>
       <c r="J106" s="49">
-        <f>MAX(0,J103+Materiales!$H$18-I105-J104)</f>
+        <f>MAX(0,ROUND(J103+Materiales!$H$18-I105-J104,4))</f>
         <v/>
       </c>
       <c r="K106" s="49">
-        <f>MAX(0,K103+Materiales!$H$18-J105-K104)</f>
+        <f>MAX(0,ROUND(K103+Materiales!$H$18-J105-K104,4))</f>
         <v/>
       </c>
       <c r="L106" s="49">
-        <f>MAX(0,L103+Materiales!$H$18-K105-L104)</f>
+        <f>MAX(0,ROUND(L103+Materiales!$H$18-K105-L104,4))</f>
         <v/>
       </c>
       <c r="M106" s="46" t="n"/>

</xml_diff>